<commit_message>
Fechando o ciclo do terraform
</commit_message>
<xml_diff>
--- a/odd-orchestrator/samples/event-storming-tuangou-project-format.xlsx
+++ b/odd-orchestrator/samples/event-storming-tuangou-project-format.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/christiano.m.almeida/produtos/odd/odd-orchestrator/samples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CF3D8C6-104E-B040-ACE3-A8A0314A6130}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9D71073-3B68-F34D-B276-0F3A3F1B178B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,9 +77,6 @@
     <t>event_stream</t>
   </si>
   <si>
-    <t>tags:(event_key:group_buying.catalog.offer.view.failure service:catalogo.oferta source:odd)</t>
-  </si>
-  <si>
     <t>Oferta (Vitrine)</t>
   </si>
   <si>
@@ -222,6 +219,9 @@
   </si>
   <si>
     <t>Duplicated event_key 'group_buying.catalog.search.view' in source rows; row 15 renamed to 'group_buying.catalog.search.view.dup2'.</t>
+  </si>
+  <si>
+    <t>tags:(event_key:group_buying.catalog.offer.view.failure)</t>
   </si>
 </sst>
 </file>
@@ -667,13 +667,13 @@
         <v>17</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="J2" s="2">
         <v>4</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="32" x14ac:dyDescent="0.2">
@@ -681,10 +681,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>21</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>13</v>
@@ -702,13 +702,13 @@
         <v>17</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J3" s="2">
         <v>5</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="48" x14ac:dyDescent="0.2">
@@ -716,34 +716,34 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>24</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>27</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J4" s="2">
         <v>8</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="48" x14ac:dyDescent="0.2">
@@ -751,34 +751,34 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="D5" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H5" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J5" s="2">
         <v>9</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="48" x14ac:dyDescent="0.2">
@@ -786,34 +786,34 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>37</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>38</v>
       </c>
       <c r="H6" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J6" s="2">
         <v>12</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="48" x14ac:dyDescent="0.2">
@@ -821,34 +821,34 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>42</v>
-      </c>
       <c r="D7" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="J7" s="2">
         <v>13</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="32" x14ac:dyDescent="0.2">
@@ -856,34 +856,34 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>46</v>
-      </c>
       <c r="D8" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>14</v>
       </c>
       <c r="F8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>47</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>48</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>17</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J8" s="2">
         <v>14</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -902,66 +902,66 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>55</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>57</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>61</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>63</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>65</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>66</v>
       </c>
     </row>
   </sheetData>

</xml_diff>